<commit_message>
modified the tasks to conference
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wen2188317/PycharmProjects/PythonProject/githubTimeline/docs/conference_timeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C54D61D-B2B9-8044-A328-18C8E35706F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30259BAA-5855-9941-B57A-B2B4F09EE233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>Task Name</t>
   </si>
@@ -40,121 +40,73 @@
     <t>Depends On</t>
   </si>
   <si>
-    <t>Define project scope</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
     <t>Alice</t>
   </si>
   <si>
-    <t>Create wireframes</t>
-  </si>
-  <si>
-    <t>Design</t>
-  </si>
-  <si>
-    <t>2025-04-17</t>
-  </si>
-  <si>
-    <t>2025-04-19</t>
-  </si>
-  <si>
     <t>Bob</t>
   </si>
   <si>
-    <t>Design UI mockups</t>
-  </si>
-  <si>
-    <t>Set up project repo</t>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>2025-04-18</t>
-  </si>
-  <si>
-    <t>Frontend development</t>
-  </si>
-  <si>
-    <t>2025-04-24</t>
-  </si>
-  <si>
-    <t>2025-04-30</t>
-  </si>
-  <si>
     <t>Charlie</t>
   </si>
   <si>
-    <t>Design UI mockups, Set up project repo</t>
-  </si>
-  <si>
-    <t>Backend development</t>
-  </si>
-  <si>
     <t>Dana</t>
   </si>
   <si>
-    <t>Integrate frontend/backend</t>
-  </si>
-  <si>
-    <t>2025-05-03</t>
-  </si>
-  <si>
-    <t>Charlie, Dana</t>
-  </si>
-  <si>
-    <t>Frontend development, Backend development</t>
-  </si>
-  <si>
-    <t>Write unit tests</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Erin</t>
-  </si>
-  <si>
-    <t>User acceptance testing</t>
-  </si>
-  <si>
-    <t>Final fixes &amp; deploy MVP</t>
-  </si>
-  <si>
-    <t>Launch</t>
-  </si>
-  <si>
     <t>Location</t>
   </si>
   <si>
-    <t>New York</t>
-  </si>
-  <si>
-    <t>Phoenix</t>
-  </si>
-  <si>
-    <t>Beijing</t>
-  </si>
-  <si>
-    <t>Shanghai</t>
-  </si>
-  <si>
-    <t>Chicago</t>
-  </si>
-  <si>
-    <t>Boston</t>
-  </si>
-  <si>
-    <t>Los Angeles</t>
-  </si>
-  <si>
-    <t>remote</t>
-  </si>
-  <si>
-    <t>Nothing</t>
+    <t>CA, U.S.</t>
+  </si>
+  <si>
+    <t>conference</t>
+  </si>
+  <si>
+    <t>International Solid-State Circuits Conference</t>
+  </si>
+  <si>
+    <t>European Solid-State Circuits Conference</t>
+  </si>
+  <si>
+    <t>Radio Frequency Integrated Circuits Symposium</t>
+  </si>
+  <si>
+    <t>Symposium on VLSI Technology and Circuits</t>
+  </si>
+  <si>
+    <t>IEEE International Symposium on Circuits and Systems</t>
+  </si>
+  <si>
+    <t>Asian Solid-State Circuits Conference</t>
+  </si>
+  <si>
+    <t>Seoul, South Korea</t>
+  </si>
+  <si>
+    <t>Kyoto, Japan</t>
+  </si>
+  <si>
+    <t>London, UK</t>
+  </si>
+  <si>
+    <t>Munich, Germany</t>
+  </si>
+  <si>
+    <t>ISSCC (DL: 9/4/24)</t>
+  </si>
+  <si>
+    <t>ESSCIRC (DL: 4/4/25)</t>
+  </si>
+  <si>
+    <t>RFIC (DL: 3/13/25)</t>
+  </si>
+  <si>
+    <t>VLSI Symosium (DL: 2/28/25)</t>
+  </si>
+  <si>
+    <t>ISCAS (DL: 10/28/24)</t>
+  </si>
+  <si>
+    <t>ASSCC (DL: 6/4/25)</t>
   </si>
 </sst>
 </file>
@@ -164,7 +116,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,6 +129,11 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="2">
@@ -225,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -236,6 +193,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,13 +499,13 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" customWidth="1"/>
     <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -570,238 +528,162 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45704</v>
+      </c>
+      <c r="D2" s="3">
+        <v>45708</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3">
+        <v>45908</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45911</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3">
-        <v>45674</v>
-      </c>
-      <c r="D2" s="3">
-        <v>45682</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3">
+        <v>45823</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45825</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3">
+        <v>45816</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45820</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3">
+        <v>45802</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45805</v>
+      </c>
+      <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3">
+        <v>45964</v>
+      </c>
+      <c r="D7" s="3">
+        <v>45967</v>
+      </c>
+      <c r="E7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3">
-        <v>45920</v>
-      </c>
-      <c r="D4" s="3">
-        <v>45923</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="F7" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="3">
-        <v>45862</v>
-      </c>
-      <c r="D6" s="3">
-        <v>45868</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="G7" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="3">
-        <v>45781</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" t="s">
-        <v>42</v>
-      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="3">
-        <v>45904</v>
-      </c>
-      <c r="D9" s="3">
-        <v>45905</v>
-      </c>
-      <c r="E9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="3">
-        <v>45870</v>
-      </c>
-      <c r="D10" s="3">
-        <v>45877</v>
-      </c>
-      <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="3">
-        <v>45969</v>
-      </c>
-      <c r="D11" s="3">
-        <v>45971</v>
-      </c>
-      <c r="E11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" t="s">
-        <v>43</v>
-      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>